<commit_message>
Développement de l'onglet debug
</commit_message>
<xml_diff>
--- a/data/Sorts.xlsx
+++ b/data/Sorts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Python\periples\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D9F632-432A-42EC-BDE8-2F2EB357D788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D032310E-26E4-4204-AE60-6CC4E4CBA432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="381">
   <si>
     <t>Nom</t>
   </si>
@@ -1005,9 +1005,6 @@
     <t>Descritption</t>
   </si>
   <si>
-    <t>1 / jour</t>
-  </si>
-  <si>
     <t>Limitation</t>
   </si>
   <si>
@@ -1035,9 +1032,6 @@
     <t>Gêles les ennemis, leur faisant perdre leur action pendant 1 tour.</t>
   </si>
   <si>
-    <t>2 / jour</t>
-  </si>
-  <si>
     <t xml:space="preserve">Inflige 6 dégats magiques à tous les adversaires. </t>
   </si>
   <si>
@@ -1120,9 +1114,6 @@
   </si>
   <si>
     <t>Utilise une ressource pour empêcher les actions de tous adversaires pendant deux tours.</t>
-  </si>
-  <si>
-    <t>3 / jour</t>
   </si>
   <si>
     <t>Ignore la parade des ennemis.</t>
@@ -1924,7 +1915,7 @@
         <v>324</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1935,10 +1926,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="I3" s="1"/>
     </row>
@@ -1950,7 +1941,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D4" s="1"/>
       <c r="I4" s="1"/>
@@ -1963,7 +1954,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D5" s="1"/>
     </row>
@@ -1975,7 +1966,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -1987,9 +1978,11 @@
         <v>1</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>331</v>
-      </c>
-      <c r="D7" s="1"/>
+        <v>330</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>338</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
@@ -1999,7 +1992,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D8" s="1"/>
     </row>
@@ -2011,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D9" s="1"/>
     </row>
@@ -2023,7 +2016,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D10" s="1"/>
     </row>
@@ -2035,10 +2028,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2049,10 +2042,10 @@
         <v>2</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2063,7 +2056,7 @@
         <v>2</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D13" s="1"/>
     </row>
@@ -2075,10 +2068,10 @@
         <v>2</v>
       </c>
       <c r="C14" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>338</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="26.25" x14ac:dyDescent="0.25">
@@ -2089,7 +2082,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D15" s="1"/>
     </row>
@@ -2101,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D16" s="1"/>
     </row>
@@ -2113,10 +2106,10 @@
         <v>1</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -2127,7 +2120,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D18" s="1"/>
     </row>
@@ -2139,10 +2132,10 @@
         <v>1</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
@@ -2153,10 +2146,10 @@
         <v>2</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -2167,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D21" s="1"/>
     </row>
@@ -2179,10 +2172,10 @@
         <v>0</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -2193,7 +2186,7 @@
         <v>0</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D23" s="1"/>
     </row>
@@ -2205,10 +2198,10 @@
         <v>0</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -2219,10 +2212,10 @@
         <v>0</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2233,10 +2226,10 @@
         <v>0</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -2247,7 +2240,7 @@
         <v>0</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D27" s="1"/>
     </row>
@@ -2259,10 +2252,10 @@
         <v>0</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2273,10 +2266,10 @@
         <v>0</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2287,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D30" s="1"/>
     </row>
@@ -2299,7 +2292,7 @@
         <v>0</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D31" s="1"/>
     </row>
@@ -2311,84 +2304,84 @@
         <v>0</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D32" s="1"/>
     </row>
     <row r="33" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B33" s="1">
         <v>1</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="B34" s="1">
         <v>1</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B35" s="1">
         <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="64.5" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="B36" s="1">
         <v>1</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B37" s="1">
         <v>2</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D37" s="1"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B38" s="1">
         <v>2</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2399,7 +2392,7 @@
         <v>0</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D39" s="1"/>
     </row>
@@ -2411,10 +2404,10 @@
         <v>0</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -2425,7 +2418,7 @@
         <v>0</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D41" s="1"/>
     </row>
@@ -2437,10 +2430,10 @@
         <v>0</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -2451,10 +2444,10 @@
         <v>0</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2465,10 +2458,10 @@
         <v>0</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -2479,7 +2472,7 @@
         <v>0</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D45" s="1"/>
     </row>
@@ -2491,10 +2484,10 @@
         <v>0</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2505,10 +2498,10 @@
         <v>0</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2519,10 +2512,10 @@
         <v>0</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2533,10 +2526,10 @@
         <v>0</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
@@ -2547,10 +2540,10 @@
         <v>0</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2561,10 +2554,10 @@
         <v>0</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2575,10 +2568,10 @@
         <v>0</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2589,10 +2582,10 @@
         <v>0</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2603,10 +2596,10 @@
         <v>0</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mise à jour du fichier excel Sorts
</commit_message>
<xml_diff>
--- a/data/Sorts.xlsx
+++ b/data/Sorts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Python\periples\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9C03F1-8CF1-4FB8-8FE9-D96DDFE47450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF30A4AE-7073-4B17-8316-F8AF0791F60A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2074,7 +2074,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>293</v>
       </c>
@@ -2117,7 +2117,7 @@
         <v>296</v>
       </c>
       <c r="B18" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>340</v>
@@ -2138,7 +2138,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>298</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>308</v>
       </c>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="D31" s="1"/>
     </row>
-    <row r="32" spans="1:4" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>310</v>
       </c>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="D32" s="1"/>
     </row>
-    <row r="33" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>378</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>376</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="39" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>379</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>311</v>
       </c>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="D41" s="1"/>
     </row>
-    <row r="42" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>314</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>316</v>
       </c>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D45" s="1"/>
     </row>
-    <row r="46" spans="1:4" ht="39" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
         <v>317</v>
       </c>
@@ -2490,7 +2490,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
         <v>319</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>320</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>321</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>322</v>
       </c>

</xml_diff>

<commit_message>
correction d'affaiblissement et d'assaut furieux
</commit_message>
<xml_diff>
--- a/data/Sorts.xlsx
+++ b/data/Sorts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Python\periples\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C935FC8-C0EA-4333-966F-548C6BE3E8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5E5AB1-D0CB-4A83-8DF1-4CE8282C4A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -416,9 +416,6 @@
     <t>Assaut furieux</t>
   </si>
   <si>
-    <t>Réussit toutes ses attaques sans laner le dé, et inflige le double de dégâts.</t>
-  </si>
-  <si>
     <t>Raishi 1</t>
   </si>
   <si>
@@ -1329,6 +1326,9 @@
   </si>
   <si>
     <t>Après une attaque réussie, bloque l'action de cet ennemi.</t>
+  </si>
+  <si>
+    <t>Réussit toutes ses attaques sans lancer le dé, et inflige le double de dégâts.</t>
   </si>
 </sst>
 </file>
@@ -2141,7 +2141,7 @@
         <v>87</v>
       </c>
       <c r="D29" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E29" t="s">
         <v>36</v>
@@ -2219,7 +2219,7 @@
         <v>104</v>
       </c>
       <c r="D35" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E35" t="s">
         <v>9</v>
@@ -2342,7 +2342,7 @@
         <v>129</v>
       </c>
       <c r="D44" t="s">
-        <v>130</v>
+        <v>434</v>
       </c>
       <c r="E44" t="s">
         <v>9</v>
@@ -2350,24 +2350,24 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>130</v>
+      </c>
+      <c r="B45" t="s">
         <v>131</v>
       </c>
-      <c r="B45" t="s">
+      <c r="D45" t="s">
         <v>132</v>
-      </c>
-      <c r="D45" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>133</v>
+      </c>
+      <c r="B46" t="s">
         <v>134</v>
       </c>
-      <c r="B46" t="s">
+      <c r="D46" t="s">
         <v>135</v>
-      </c>
-      <c r="D46" t="s">
-        <v>136</v>
       </c>
       <c r="E46" t="s">
         <v>36</v>
@@ -2375,13 +2375,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>136</v>
+      </c>
+      <c r="B47" t="s">
         <v>137</v>
       </c>
-      <c r="B47" t="s">
+      <c r="D47" t="s">
         <v>138</v>
-      </c>
-      <c r="D47" t="s">
-        <v>139</v>
       </c>
       <c r="E47" t="s">
         <v>9</v>
@@ -2389,13 +2389,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" t="s">
         <v>140</v>
       </c>
-      <c r="B48" t="s">
+      <c r="D48" t="s">
         <v>141</v>
-      </c>
-      <c r="D48" t="s">
-        <v>142</v>
       </c>
       <c r="E48" t="s">
         <v>75</v>
@@ -2403,13 +2403,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>142</v>
+      </c>
+      <c r="B49" t="s">
         <v>143</v>
       </c>
-      <c r="B49" t="s">
+      <c r="D49" t="s">
         <v>144</v>
-      </c>
-      <c r="D49" t="s">
-        <v>145</v>
       </c>
       <c r="E49" t="s">
         <v>75</v>
@@ -2417,13 +2417,13 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>145</v>
+      </c>
+      <c r="B50" t="s">
         <v>146</v>
       </c>
-      <c r="B50" t="s">
+      <c r="D50" t="s">
         <v>147</v>
-      </c>
-      <c r="D50" t="s">
-        <v>148</v>
       </c>
       <c r="E50" t="s">
         <v>9</v>
@@ -2431,13 +2431,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>148</v>
+      </c>
+      <c r="B51" t="s">
         <v>149</v>
       </c>
-      <c r="B51" t="s">
+      <c r="D51" t="s">
         <v>150</v>
-      </c>
-      <c r="D51" t="s">
-        <v>151</v>
       </c>
       <c r="E51" t="s">
         <v>23</v>
@@ -2445,13 +2445,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>151</v>
+      </c>
+      <c r="B52" t="s">
         <v>152</v>
       </c>
-      <c r="B52" t="s">
+      <c r="D52" t="s">
         <v>153</v>
-      </c>
-      <c r="D52" t="s">
-        <v>154</v>
       </c>
       <c r="E52" t="s">
         <v>36</v>
@@ -2476,30 +2476,30 @@
   <sheetData>
     <row r="1" spans="1:6" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="C2" s="1">
         <v>6</v>
@@ -2516,10 +2516,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="C3" s="1">
         <v>0</v>
@@ -2536,10 +2536,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>165</v>
       </c>
       <c r="C4" s="1">
         <v>3</v>
@@ -2556,10 +2556,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="C5" s="1">
         <v>5</v>
@@ -2576,10 +2576,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="C6" s="1">
         <v>3</v>
@@ -2596,10 +2596,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>171</v>
       </c>
       <c r="C7" s="1">
         <v>5</v>
@@ -2616,10 +2616,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="C8" s="1">
         <v>5</v>
@@ -2636,10 +2636,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>175</v>
       </c>
       <c r="C9" s="1">
         <v>6</v>
@@ -2656,10 +2656,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C10" s="1">
         <v>4</v>
@@ -2676,10 +2676,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C11" s="1">
         <v>6</v>
@@ -2696,10 +2696,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="C12" s="1">
         <v>4</v>
@@ -2716,10 +2716,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="C13" s="1">
         <v>6</v>
@@ -2754,36 +2754,36 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>185</v>
-      </c>
       <c r="G1" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="C2" s="1">
         <v>2</v>
@@ -2806,10 +2806,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>188</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>189</v>
       </c>
       <c r="C3" s="1">
         <v>0</v>
@@ -2832,10 +2832,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
@@ -2858,10 +2858,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>192</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>193</v>
       </c>
       <c r="C5" s="1">
         <v>1</v>
@@ -2884,10 +2884,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>194</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>195</v>
       </c>
       <c r="C6" s="1">
         <v>2</v>
@@ -2910,10 +2910,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>197</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
@@ -2936,10 +2936,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>198</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>199</v>
       </c>
       <c r="C8" s="1">
         <v>3</v>
@@ -2962,10 +2962,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -2988,10 +2988,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>202</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>203</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
@@ -3014,10 +3014,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>205</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
@@ -3040,10 +3040,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
@@ -3066,10 +3066,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>207</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>208</v>
       </c>
       <c r="C13" s="1">
         <v>0</v>
@@ -3092,10 +3092,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C14" s="1">
         <v>0</v>
@@ -3118,10 +3118,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C15" s="1">
         <v>2</v>
@@ -3144,10 +3144,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
@@ -3170,10 +3170,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C17" s="1">
         <v>2</v>
@@ -3196,10 +3196,10 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>213</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>214</v>
       </c>
       <c r="C18" s="1">
         <v>1</v>
@@ -3222,10 +3222,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C19" s="1">
         <v>1</v>
@@ -3248,10 +3248,10 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>216</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>217</v>
       </c>
       <c r="C20" s="1">
         <v>2</v>
@@ -3274,10 +3274,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>218</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>219</v>
       </c>
       <c r="C21" s="1">
         <v>3</v>
@@ -3300,10 +3300,10 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C22" s="1">
         <v>1</v>
@@ -3326,10 +3326,10 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>221</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>222</v>
       </c>
       <c r="C23" s="1">
         <v>1</v>
@@ -3352,10 +3352,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="C24" s="1">
         <v>3</v>
@@ -3378,10 +3378,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C25" s="1">
         <v>2</v>
@@ -3404,10 +3404,10 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C26" s="1">
         <v>2</v>
@@ -3430,10 +3430,10 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C27" s="1">
         <v>0</v>
@@ -3456,10 +3456,10 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>228</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>229</v>
       </c>
       <c r="C28" s="1">
         <v>0</v>
@@ -3482,10 +3482,10 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>230</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>231</v>
       </c>
       <c r="C29" s="1">
         <v>0</v>
@@ -3508,10 +3508,10 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C30" s="1">
         <v>0</v>
@@ -3534,10 +3534,10 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C31" s="1">
         <v>0</v>
@@ -3560,10 +3560,10 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C32" s="1">
         <v>0</v>
@@ -3586,10 +3586,10 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C33" s="1">
         <v>0</v>
@@ -3612,10 +3612,10 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>236</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>237</v>
       </c>
       <c r="C34" s="1">
         <v>0</v>
@@ -3638,10 +3638,10 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C35" s="1">
         <v>0</v>
@@ -3664,10 +3664,10 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>239</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>240</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>
@@ -3690,10 +3690,10 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>241</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>242</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
@@ -3716,10 +3716,10 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>243</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>244</v>
       </c>
       <c r="C38" s="1">
         <v>2</v>
@@ -3742,10 +3742,10 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>245</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>246</v>
       </c>
       <c r="C39" s="1">
         <v>0</v>
@@ -3768,10 +3768,10 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B40" s="6" t="s">
         <v>247</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>248</v>
       </c>
       <c r="C40" s="1">
         <v>0</v>
@@ -3794,10 +3794,10 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B41" s="6" t="s">
         <v>249</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>250</v>
       </c>
       <c r="C41" s="1">
         <v>4</v>
@@ -3820,10 +3820,10 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>251</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>252</v>
       </c>
       <c r="C42" s="1">
         <v>0</v>
@@ -3846,10 +3846,10 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>253</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>254</v>
       </c>
       <c r="C43" s="1">
         <v>0</v>
@@ -3872,10 +3872,10 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B44" s="6" t="s">
         <v>255</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>256</v>
       </c>
       <c r="C44" s="1">
         <v>2</v>
@@ -3898,10 +3898,10 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="B45" s="6" t="s">
         <v>257</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>258</v>
       </c>
       <c r="C45" s="1">
         <v>0</v>
@@ -3924,10 +3924,10 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="B46" s="6" t="s">
         <v>259</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>260</v>
       </c>
       <c r="C46" s="1">
         <v>4</v>
@@ -3950,10 +3950,10 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>261</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>262</v>
       </c>
       <c r="C47" s="1">
         <v>0</v>
@@ -3976,10 +3976,10 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="B48" s="6" t="s">
         <v>263</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>264</v>
       </c>
       <c r="C48" s="1">
         <v>2</v>
@@ -4002,10 +4002,10 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B49" s="6" t="s">
         <v>265</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>266</v>
       </c>
       <c r="C49" s="1">
         <v>3</v>
@@ -4028,10 +4028,10 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="B50" s="6" t="s">
         <v>267</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>268</v>
       </c>
       <c r="C50" s="1">
         <v>0</v>
@@ -4054,10 +4054,10 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>269</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>270</v>
       </c>
       <c r="C51" s="1">
         <v>3</v>
@@ -4080,10 +4080,10 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>271</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>272</v>
       </c>
       <c r="C52" s="1">
         <v>0</v>
@@ -4106,10 +4106,10 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>273</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>274</v>
       </c>
       <c r="C53" s="1">
         <v>0</v>
@@ -4155,54 +4155,54 @@
   <sheetData>
     <row r="1" spans="1:14" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>285</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>287</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>288</v>
       </c>
       <c r="C2" s="6">
         <v>10</v>
@@ -4235,18 +4235,18 @@
         <v>2</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>290</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>291</v>
       </c>
       <c r="C3" s="6">
         <v>12</v>
@@ -4279,18 +4279,18 @@
         <v>2</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>292</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>293</v>
       </c>
       <c r="C4" s="6">
         <v>10</v>
@@ -4323,18 +4323,18 @@
         <v>1</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>294</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>295</v>
       </c>
       <c r="C5" s="6">
         <v>11</v>
@@ -4367,18 +4367,18 @@
         <v>1</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>296</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>297</v>
       </c>
       <c r="C6" s="6">
         <v>12</v>
@@ -4411,18 +4411,18 @@
         <v>1</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>298</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>299</v>
       </c>
       <c r="C7" s="6">
         <v>14</v>
@@ -4455,18 +4455,18 @@
         <v>0</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>301</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>302</v>
       </c>
       <c r="C8" s="6">
         <v>12</v>
@@ -4499,18 +4499,18 @@
         <v>2</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>303</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>304</v>
       </c>
       <c r="C9" s="6">
         <v>12</v>
@@ -4543,18 +4543,18 @@
         <v>0</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>305</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>306</v>
       </c>
       <c r="C10" s="6">
         <v>10</v>
@@ -4587,18 +4587,18 @@
         <v>1</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>307</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>308</v>
       </c>
       <c r="C11" s="6">
         <v>13</v>
@@ -4631,18 +4631,18 @@
         <v>1</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>309</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>310</v>
       </c>
       <c r="C12" s="6">
         <v>12</v>
@@ -4675,18 +4675,18 @@
         <v>1</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>311</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>312</v>
       </c>
       <c r="C13" s="6">
         <v>13</v>
@@ -4719,18 +4719,18 @@
         <v>1</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>313</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>314</v>
       </c>
       <c r="C14" s="6">
         <v>12</v>
@@ -4763,18 +4763,18 @@
         <v>1</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>315</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>316</v>
       </c>
       <c r="C15" s="6">
         <v>13</v>
@@ -4807,18 +4807,18 @@
         <v>1</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>317</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>318</v>
       </c>
       <c r="C16" s="6">
         <v>14</v>
@@ -4851,18 +4851,18 @@
         <v>1</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>319</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>320</v>
       </c>
       <c r="C17" s="6">
         <v>14</v>
@@ -4895,18 +4895,18 @@
         <v>0</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>321</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>322</v>
       </c>
       <c r="C18" s="6">
         <v>13</v>
@@ -4939,18 +4939,18 @@
         <v>0</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>323</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>324</v>
       </c>
       <c r="C19" s="6">
         <v>12</v>
@@ -4983,18 +4983,18 @@
         <v>2</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>325</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>326</v>
       </c>
       <c r="C20" s="6">
         <v>14</v>
@@ -5027,18 +5027,18 @@
         <v>0</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>328</v>
       </c>
       <c r="C21" s="6">
         <v>12</v>
@@ -5071,18 +5071,18 @@
         <v>1</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>329</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>330</v>
       </c>
       <c r="C22" s="6">
         <v>14</v>
@@ -5115,18 +5115,18 @@
         <v>1</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>331</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>332</v>
       </c>
       <c r="C23" s="6">
         <v>13</v>
@@ -5159,18 +5159,18 @@
         <v>1</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>333</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>334</v>
       </c>
       <c r="C24" s="6">
         <v>14</v>
@@ -5203,18 +5203,18 @@
         <v>2</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>335</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>336</v>
       </c>
       <c r="C25" s="6">
         <v>13</v>
@@ -5247,18 +5247,18 @@
         <v>2</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>337</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>338</v>
       </c>
       <c r="C26" s="6">
         <v>12</v>
@@ -5291,18 +5291,18 @@
         <v>2</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>339</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>340</v>
       </c>
       <c r="C27" s="6">
         <v>14</v>
@@ -5335,18 +5335,18 @@
         <v>3</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>341</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>342</v>
       </c>
       <c r="C28" s="6">
         <v>15</v>
@@ -5379,18 +5379,18 @@
         <v>2</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>343</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>344</v>
       </c>
       <c r="C29" s="6">
         <v>11</v>
@@ -5423,18 +5423,18 @@
         <v>3</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>345</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>346</v>
       </c>
       <c r="C30" s="6">
         <v>10</v>
@@ -5467,18 +5467,18 @@
         <v>3</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>347</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>348</v>
       </c>
       <c r="C31" s="6">
         <v>14</v>
@@ -5511,18 +5511,18 @@
         <v>2</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="B32" s="6" t="s">
         <v>349</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>350</v>
       </c>
       <c r="C32" s="6">
         <v>12</v>
@@ -5555,18 +5555,18 @@
         <v>2</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>351</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>352</v>
       </c>
       <c r="C33" s="6">
         <v>15</v>
@@ -5599,18 +5599,18 @@
         <v>2</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>353</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>354</v>
       </c>
       <c r="C34" s="6">
         <v>13</v>
@@ -5643,18 +5643,18 @@
         <v>2</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>355</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>356</v>
       </c>
       <c r="C35" s="6">
         <v>15</v>
@@ -5687,18 +5687,18 @@
         <v>2</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>357</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>358</v>
       </c>
       <c r="C36" s="6">
         <v>14</v>
@@ -5731,18 +5731,18 @@
         <v>2</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>359</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>360</v>
       </c>
       <c r="C37" s="6">
         <v>12</v>
@@ -5775,18 +5775,18 @@
         <v>2</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>361</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>362</v>
       </c>
       <c r="C38" s="6">
         <v>14</v>
@@ -5819,18 +5819,18 @@
         <v>2</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>363</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>364</v>
       </c>
       <c r="C39" s="6">
         <v>13</v>
@@ -5863,18 +5863,18 @@
         <v>2</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="B40" s="6" t="s">
         <v>365</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>366</v>
       </c>
       <c r="C40" s="6">
         <v>14</v>
@@ -5907,18 +5907,18 @@
         <v>3</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B41" s="6" t="s">
         <v>367</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>368</v>
       </c>
       <c r="C41" s="6">
         <v>16</v>
@@ -5951,18 +5951,18 @@
         <v>3</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>369</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>370</v>
       </c>
       <c r="C42" s="6">
         <v>16</v>
@@ -5995,18 +5995,18 @@
         <v>3</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>371</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>372</v>
       </c>
       <c r="C43" s="6">
         <v>14</v>
@@ -6039,18 +6039,18 @@
         <v>4</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B44" s="6" t="s">
         <v>373</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>374</v>
       </c>
       <c r="C44" s="6">
         <v>12</v>
@@ -6083,18 +6083,18 @@
         <v>0</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="B45" s="6" t="s">
         <v>375</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>376</v>
       </c>
       <c r="C45" s="6">
         <v>12</v>
@@ -6127,18 +6127,18 @@
         <v>2</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="B46" s="6" t="s">
         <v>377</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>378</v>
       </c>
       <c r="C46" s="6">
         <v>13</v>
@@ -6171,18 +6171,18 @@
         <v>2</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>379</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>380</v>
       </c>
       <c r="C47" s="6">
         <v>14</v>
@@ -6215,18 +6215,18 @@
         <v>2</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="B48" s="6" t="s">
         <v>381</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>382</v>
       </c>
       <c r="C48" s="6">
         <v>11</v>
@@ -6259,18 +6259,18 @@
         <v>2</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="B49" s="6" t="s">
         <v>383</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>384</v>
       </c>
       <c r="C49" s="6">
         <v>10</v>
@@ -6303,18 +6303,18 @@
         <v>2</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="B50" s="6" t="s">
         <v>385</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>386</v>
       </c>
       <c r="C50" s="6">
         <v>12</v>
@@ -6347,18 +6347,18 @@
         <v>1</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>387</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>388</v>
       </c>
       <c r="C51" s="6">
         <v>11</v>
@@ -6391,18 +6391,18 @@
         <v>1</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>389</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>390</v>
       </c>
       <c r="C52" s="6">
         <v>13</v>
@@ -6435,18 +6435,18 @@
         <v>1</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>391</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>392</v>
       </c>
       <c r="C53" s="6">
         <v>10</v>
@@ -6479,18 +6479,18 @@
         <v>1</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="B54" s="6" t="s">
         <v>393</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>394</v>
       </c>
       <c r="C54" s="6">
         <v>14</v>
@@ -6523,18 +6523,18 @@
         <v>2</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="B55" s="6" t="s">
         <v>395</v>
-      </c>
-      <c r="B55" s="6" t="s">
-        <v>396</v>
       </c>
       <c r="C55" s="6">
         <v>14</v>
@@ -6567,18 +6567,18 @@
         <v>2</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="B56" s="6" t="s">
         <v>397</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>398</v>
       </c>
       <c r="C56" s="6">
         <v>13</v>
@@ -6611,18 +6611,18 @@
         <v>2</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="B57" s="6" t="s">
         <v>399</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>400</v>
       </c>
       <c r="C57" s="6">
         <v>12</v>
@@ -6655,18 +6655,18 @@
         <v>2</v>
       </c>
       <c r="M57" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B58" s="6" t="s">
         <v>401</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>402</v>
       </c>
       <c r="C58" s="6">
         <v>15</v>
@@ -6699,18 +6699,18 @@
         <v>2</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="B59" s="6" t="s">
         <v>403</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>404</v>
       </c>
       <c r="C59" s="6">
         <v>12</v>
@@ -6743,18 +6743,18 @@
         <v>2</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="B60" s="6" t="s">
         <v>405</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>406</v>
       </c>
       <c r="C60" s="6">
         <v>14</v>
@@ -6787,18 +6787,18 @@
         <v>2</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="B61" s="6" t="s">
         <v>407</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>408</v>
       </c>
       <c r="C61" s="6">
         <v>16</v>
@@ -6831,18 +6831,18 @@
         <v>2</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>409</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>410</v>
       </c>
       <c r="C62" s="6">
         <v>14</v>
@@ -6875,18 +6875,18 @@
         <v>0</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="B63" s="6" t="s">
         <v>411</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>412</v>
       </c>
       <c r="C63" s="6">
         <v>14</v>
@@ -6919,18 +6919,18 @@
         <v>4</v>
       </c>
       <c r="M63" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="B64" s="6" t="s">
         <v>413</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>414</v>
       </c>
       <c r="C64" s="6">
         <v>14</v>
@@ -6963,18 +6963,18 @@
         <v>2</v>
       </c>
       <c r="M64" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B65" s="6" t="s">
         <v>415</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>416</v>
       </c>
       <c r="C65" s="6">
         <v>16</v>
@@ -7007,18 +7007,18 @@
         <v>3</v>
       </c>
       <c r="M65" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="B66" s="6" t="s">
         <v>417</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>418</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="1">
@@ -7034,18 +7034,18 @@
       </c>
       <c r="L66" s="5"/>
       <c r="M66" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B67" s="6" t="s">
         <v>419</v>
-      </c>
-      <c r="B67" s="6" t="s">
-        <v>420</v>
       </c>
       <c r="C67" s="6">
         <v>12</v>
@@ -7078,18 +7078,18 @@
         <v>3</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="B68" s="6" t="s">
         <v>421</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>422</v>
       </c>
       <c r="C68" s="6">
         <v>15</v>
@@ -7122,18 +7122,18 @@
         <v>4</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>423</v>
-      </c>
-      <c r="B69" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C69" s="6">
         <v>12</v>
@@ -7166,18 +7166,18 @@
         <v>2</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B70" s="6" t="s">
         <v>425</v>
-      </c>
-      <c r="B70" s="6" t="s">
-        <v>426</v>
       </c>
       <c r="C70" s="6">
         <v>16</v>
@@ -7210,18 +7210,18 @@
         <v>6</v>
       </c>
       <c r="M70" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B71" s="6" t="s">
         <v>427</v>
-      </c>
-      <c r="B71" s="6" t="s">
-        <v>428</v>
       </c>
       <c r="C71" s="6">
         <v>15</v>
@@ -7254,18 +7254,18 @@
         <v>4</v>
       </c>
       <c r="M71" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B72" s="6" t="s">
         <v>429</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>430</v>
       </c>
       <c r="C72" s="6">
         <v>18</v>
@@ -7298,18 +7298,18 @@
         <v>4</v>
       </c>
       <c r="M72" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="B73" s="6" t="s">
         <v>431</v>
-      </c>
-      <c r="B73" s="6" t="s">
-        <v>432</v>
       </c>
       <c r="C73" s="6">
         <v>16</v>
@@ -7342,10 +7342,10 @@
         <v>4</v>
       </c>
       <c r="M73" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>